<commit_message>
Publish verified live curriculum review and detailed correction report
</commit_message>
<xml_diff>
--- a/public/documents/doi-chieu-sgk-lop-4.xlsx
+++ b/public/documents/doi-chieu-sgk-lop-4.xlsx
@@ -404,11 +404,8 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B4"/>
   <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="15.83203125" customWidth="1"/>
-    <col min="3" max="3" width="80.83203125" customWidth="1"/>
-    <col min="4" max="4" width="80.83203125" customWidth="1"/>
-    <col min="5" max="5" width="22.83203125" customWidth="1"/>
+    <col min="1" max="1" width="25.83203125" customWidth="1"/>
+    <col min="2" max="2" width="130.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -424,15 +421,15 @@
         <v>Đã đối chiếu</v>
       </c>
       <c r="B2" t="str">
-        <v>Mục lục sáu sách lớp 4, lịch Tiếng Việt 35 tuần và dữ liệu luyện viết trong mã.</v>
+        <v>Mục lục sáu sách lớp 4, lịch Tiếng Việt 35 tuần, dữ liệu luyện viết và bản chụp 213 bộ công khai, 2.143 câu hỏi ngày 15/10/2026.</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Chưa kiểm tra</v>
+        <v>Ngân hàng công khai</v>
       </c>
       <c r="B3" t="str">
-        <v>Ngân hàng Firestore không đọc được: HTTP 429 Quota exceeded. Chưa xác nhận mọi câu hỏi/đáp án.</v>
+        <v>Đã sửa/bổ sung 76 câu trong 60 bản công khai và 48 câu gốc còn lưu; tải báo cáo chi tiết riêng. Chưa xác nhận các bộ riêng chưa đọc hoặc thay đổi sau thời điểm rà soát.</v>
       </c>
     </row>
     <row r="4">
@@ -453,13 +450,6 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G36"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="15.83203125" customWidth="1"/>
-    <col min="3" max="3" width="80.83203125" customWidth="1"/>
-    <col min="4" max="4" width="80.83203125" customWidth="1"/>
-    <col min="5" max="5" width="22.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1299,13 +1289,6 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E74"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="15.83203125" customWidth="1"/>
-    <col min="3" max="3" width="80.83203125" customWidth="1"/>
-    <col min="4" max="4" width="80.83203125" customWidth="1"/>
-    <col min="5" max="5" width="22.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2575,13 +2558,6 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E32"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="15.83203125" customWidth="1"/>
-    <col min="3" max="3" width="80.83203125" customWidth="1"/>
-    <col min="4" max="4" width="80.83203125" customWidth="1"/>
-    <col min="5" max="5" width="22.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3137,13 +3113,6 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E28"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="15.83203125" customWidth="1"/>
-    <col min="3" max="3" width="80.83203125" customWidth="1"/>
-    <col min="4" max="4" width="80.83203125" customWidth="1"/>
-    <col min="5" max="5" width="22.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3631,13 +3600,6 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D36"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="15.83203125" customWidth="1"/>
-    <col min="3" max="3" width="80.83203125" customWidth="1"/>
-    <col min="4" max="4" width="80.83203125" customWidth="1"/>
-    <col min="5" max="5" width="22.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">

</xml_diff>